<commit_message>
Add Role (front-end/back-end) and Token consumption tier columns
Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/agentic_ai_banking_payments.xlsx
+++ b/data/agentic_ai_banking_payments.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -715,6 +715,58 @@
         </is>
       </c>
       <c r="C20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Role: Front-end</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Agent interacts directly with external counterparties — retail or wholesale customers, merchants, dealers, or third-party AI surfaces (e.g., ChatGPT). Drives revenue, CX or distribution.</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Role: Back-end</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Agent runs inside the institution — employee productivity, ops, compliance, software engineering, treasury, finance, risk. Drives cost, throughput or control.</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Role: Both</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Same product line spans customer-facing and internal-facing surfaces (e.g., a contact-centre platform that powers both bot self-service and agent assist).</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Token consumption tiers</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Qualitative monthly token-usage estimate based on scale (users × interactions × avg tokens). Buckets: Very High (&gt;1B tokens/mo), High (100M–1B), Medium (10M–100M), Low (&lt;10M), N/A (not LLM-based or pure infra), N/D (not disclosed). Estimates are illustrative — vendors rarely publish exact figures.</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -727,19 +779,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="59" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
     <col width="60" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="49" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -765,30 +819,40 @@
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
+          <t>Role (Front-end / Back-end)</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
           <t>Underlying models / partners</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Stage (2026)</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Scale / Adoption</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Reported impact</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>Token consumption (tier)</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Announced</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>Source ID</t>
         </is>
@@ -817,30 +881,40 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>Back-end</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>OpenAI, Anthropic (multi-model)</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>In production</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>230k–250k employees with access (~50% daily); 450+ agentic use cases live, target 1,000</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>3–6 hrs/week saved per user; Nvidia IB deck generated in ~30s; $18B annual tech budget supports build</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Very High</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>2024-2026</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
@@ -869,30 +943,40 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
+          <t>Back-end</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
           <t>Internal NLP + LLM Suite</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>In production</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Bank-wide in commercial banking</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>~360,000 lawyer/analyst hours saved per year; 150+ data attributes extracted</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>2017 (re-platformed 2025-26)</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
@@ -921,30 +1005,40 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
           <t>Proprietary small language model + NLU</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>In production</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>42M consumers, 40k business clients, 95% of 213k staff</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>~2M interactions/day; work equivalent of ~11,000 FTE</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Low (small model, intent classifier)</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>2018 (continual)</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
@@ -973,30 +1067,40 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
+          <t>Both (employee assist + client-facing answers)</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
           <t>Internal genAI + Azure OpenAI</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>In production</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Global Payments Solutions client teams</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Faster RFP / payments-product responses; part of $4B 2025 AI budget</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>Sep-2025</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
@@ -1025,30 +1129,40 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
+          <t>Back-end</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
           <t>Google Gemini, Anthropic Claude</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Pilot → staged rollout</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>5,000-user pilot then thousands more across firm</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Compresses multi-step research into single prompts; example: top-5 branded card analysis + Spanish translation in one prompt</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>Sep-2025</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>S3</t>
         </is>
@@ -1077,30 +1191,40 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
+          <t>Back-end</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
           <t>GPT-5, Gemini, Claude, Llama (router)</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>In production</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>~10k pilot Jan-2025; firm-wide June-2025</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Routes prompts to best-fit model in firewalled environment</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Jun-2025</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>S4</t>
         </is>
@@ -1129,30 +1253,40 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
+          <t>Back-end</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
           <t>Cognition Devin</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>In production</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>12,000 developers</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Reported 3-4x productivity vs. previous tools</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Very High (long-horizon coding agent runs)</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>S4</t>
         </is>
@@ -1181,30 +1315,40 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
+          <t>Back-end</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
           <t>Anthropic Claude Opus 4.6</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Production rollout</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Touches portion of $2.5T AUS; embedded Anthropic engineers</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>First major bank deploying autonomous agents in trade ops</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Very High (trade-ops + surveillance volume)</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>Feb-2026</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>S4, S20</t>
         </is>
@@ -1233,30 +1377,40 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
+          <t>Back-end</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
           <t>Internal</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>In production</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Investment banking division</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Pairs deal-makers with internal expertise for complex deals</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>S4</t>
         </is>
@@ -1285,30 +1439,40 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
+          <t>Back-end (advisor-facing)</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
           <t>OpenAI GPT-4 family</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>In production</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>98% of advisor teams adopted; ~15k advisors</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Standardises advisor research access</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2023-2024</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>S5</t>
         </is>
@@ -1337,30 +1501,40 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
+          <t>Back-end (advisor-facing)</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
           <t>OpenAI Whisper + GPT-4</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>In production</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Wealth advisors firm-wide; ~1M Zoom calls/year</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>~30 min saved per meeting; auto-drafts saved to Salesforce</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>High (1M call transcripts/yr)</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>Jul-2024</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>S5</t>
         </is>
@@ -1389,30 +1563,40 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
+          <t>Front-end</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
           <t>Google Cloud (PaLM/Gemini)</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>In production</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Mobile-app users</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>30-day balance / 14-day txn forecasts; subscription tracking</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>2023 (expanded 2026)</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>S6</t>
         </is>
@@ -1441,30 +1625,40 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
           <t>Google Agentspace, NotebookLM, Deep Research</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Bank-wide rollout</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>215,000 employees in scope</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>Custom agents query ~250k vendor contracts; automates routine service</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Very High (215k seats + customer agents)</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>S6</t>
         </is>
@@ -1493,30 +1687,40 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
           <t>Multi-vendor (incl. Google Cloud, Microsoft)</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Scaling</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Global trade finance + retail divisions</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>Framework of tiered autonomy with human oversight</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>S7</t>
         </is>
@@ -1545,30 +1749,40 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
+          <t>Both (BarxBot front-end on FX; colleague assistant back-end)</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
           <t>Internal + partners</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>In production</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Barclays UK call centres; Markets FX desks</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>Reduced call handling times; emerging agentic patterns being deployed</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>2025-2026</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>S7</t>
         </is>
@@ -1597,30 +1811,40 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
           <t>Multi-model</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Scaling</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>300+ AI use cases launched 2025; new Chief AI Officer Jan-2026</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>Architectural shifts: agent marketplaces, multi-agent systems</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>2025-2026</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>S8</t>
         </is>
@@ -1649,30 +1873,40 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
+          <t>Back-end</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
           <t>Multi-vendor</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Scaling pilots</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Investment banking &amp; cross-border payments</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>Coordination layer maintains audit trail</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>S8</t>
         </is>
@@ -1701,30 +1935,40 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
+          <t>Front-end</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
           <t>Internal + partners</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>Customer rollout in 2026</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>Retail customer base</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>Targets &gt;£100M ($127M) 2026 value; 50+ GenAI solutions live</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>S9</t>
         </is>
@@ -1753,30 +1997,40 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
+          <t>Front-end</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Q1-2026 rollout to 25k customers</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>25,000 customers initial; voice-to-voice + agentic fraud later 2026</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>£1.2B AI invest in 2025; 10x productivity in financial-crime ops; 70k staff hours saved</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Medium (will scale to High with voice GA)</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>Q1-2026</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>S9</t>
         </is>
@@ -1805,30 +2059,40 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>Scaling 2026-27</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>~15k licenses → 30k (15% of workforce)</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>Targets €1B AI value by 2028; mandatory AI training 2026</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Very High</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
         <is>
           <t>2025-2026</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="L21" s="2" t="inlineStr">
         <is>
           <t>S9</t>
         </is>
@@ -1857,30 +2121,40 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>120,000 employees across 25 countries</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>83% weekly active in pilot; 20k+ custom GPTs; ~3 hrs/week saved</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr">
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Very High (120k seats + Blue customer agent)</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
         <is>
           <t>Dec-2025</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="L22" s="2" t="inlineStr">
         <is>
           <t>S10</t>
         </is>
@@ -1909,30 +2183,40 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
+          <t>Front-end</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
           <t>Internal + partners</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>Launch 2026 (NL, DE)</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>Retail mortgage customers in NL/DE first</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="I23" s="2" t="inlineStr">
         <is>
           <t>Eliminates need to talk to staff; ~€350M cost saves; 1,250 ops job exits</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr">
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>High (multi-step workflow per applicant)</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="L23" s="2" t="inlineStr">
         <is>
           <t>S11</t>
         </is>
@@ -1961,30 +2245,40 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
+          <t>Front-end</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
           <t>Internal + partners</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>Live in ES, DE</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>Call centres</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>Routine queries handled autonomously</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
+      <c r="L24" s="2" t="inlineStr">
         <is>
           <t>S11</t>
         </is>
@@ -2013,30 +2307,40 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
+          <t>Both (Joy front-end; CodeBuddy back-end)</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
           <t>Internal LLMs + partners</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>In production</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>20k+ corporate/SME customers using Joy</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="I25" s="2" t="inlineStr">
         <is>
           <t>+23% CSAT; 20% time saved on coding; AI generated ~S$1B value FY25</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr">
+      <c r="L25" s="2" t="inlineStr">
         <is>
           <t>S12</t>
         </is>
@@ -2065,30 +2369,40 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
           <t>Cohere</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>Scaling</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>Bank-wide; new dedicated AI Group reporting to CEO</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>Targets up to C$1B AI value by 2027</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>Feb-2026</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="L26" s="2" t="inlineStr">
         <is>
           <t>S13</t>
         </is>
@@ -2117,30 +2431,40 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
+          <t>Back-end</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
           <t>Multi-vendor</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>Scaling</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>Enterprise back office</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="I27" s="2" t="inlineStr">
         <is>
           <t>Part of plan to cut C$2-2.5B expenses; Vector Institute training partnership</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
+      <c r="L27" s="2" t="inlineStr">
         <is>
           <t>S13</t>
         </is>
@@ -2169,30 +2493,40 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
+          <t>Front-end (offer surface)</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
           <t>Internal</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>In production</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>Scene+ loyalty members</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>+18% YoY redemption rate</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Low (recommendation models, limited LLM tokens)</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="L28" s="2" t="inlineStr">
         <is>
           <t>S13</t>
         </is>
@@ -2221,30 +2555,40 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
+          <t>Front-end</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
           <t>NVIDIA stack + internal</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>In production</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>Dealer network customers</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="I29" s="2" t="inlineStr">
         <is>
           <t>Multi-agent system with master orchestrator; 24/7 service</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Medium (dealer-network scale)</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
         <is>
           <t>2025-2026</t>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr">
+      <c r="L29" s="2" t="inlineStr">
         <is>
           <t>S14</t>
         </is>
@@ -2273,30 +2617,40 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
+          <t>Front-end (developer / partner facing)</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
           <t>Internal</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>Live (agentic features planned)</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>Embedded-banking partners</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="I30" s="2" t="inlineStr">
         <is>
           <t>Helps biz clients discover/implement APIs; agentic features on roadmap</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr">
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
         <is>
           <t>Oct-2025</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr">
+      <c r="L30" s="2" t="inlineStr">
         <is>
           <t>S15</t>
         </is>
@@ -2325,30 +2679,40 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
+          <t>Back-end (delivered to clients)</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
           <t>Internal + partners</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>Commercial / corporate clients</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>Auto-matches payments to invoices; reduces exceptions</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr">
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
         <is>
           <t>Feb-2026</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr">
+      <c r="L31" s="2" t="inlineStr">
         <is>
           <t>S15</t>
         </is>
@@ -2377,30 +2741,40 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
+          <t>Back-end (treasury workflow)</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
           <t>Internal + partners</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>Treasury clients</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>Predictive + prescriptive automation of treasury actions</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr">
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr">
+      <c r="L32" s="2" t="inlineStr">
         <is>
           <t>S15</t>
         </is>
@@ -2417,7 +2791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -2425,10 +2799,12 @@
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="35" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="39" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="55" customWidth="1" min="9" max="9"/>
+    <col width="39" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2449,30 +2825,40 @@
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
+          <t>Role (Front-end / Back-end)</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
           <t>Supported protocols</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Key partners</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Stage (2026)</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Notable details</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Token consumption (tier)</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Announced</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Source ID</t>
         </is>
@@ -2496,30 +2882,40 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>Front-end (rails consumed by external AI agents)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>Visa Trusted Agent Protocol; supports MPP, ACP, UCP</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>AWS, Aldar, Firmly, Nekuda, Fiserv</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Launched Apr-2026</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Tokenises card numbers; verifies agent obeys consumer instructions; routes across networks</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>N/A (infrastructure; tokens consumed by partner LLMs)</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Apr-2026</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>S16</t>
         </is>
@@ -2543,30 +2939,40 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>Front-end (powers AI checkout) + Back-end (dispute audit)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
           <t>Open agent framework</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Fiserv (US merchant integration), 4,000+ advisors</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Launched Q2-2026</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Cryptographic audit trail linking identity, instructions, outcome; integrated with Fiserv merchant base</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>N/A (infra) + Low for Verifiable Intent reasoning</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Jan-2026 (suite); Q2-2026 (Agent Pay)</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>S16</t>
         </is>
@@ -2590,30 +2996,40 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
+          <t>Front-end (issuer rails for external AI agents)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
           <t>Industry-standard tokens</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>AI platform partners (unnamed)</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Launched Apr-2026</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Five components: agent registration, account enablement, purchase intent, tokenised credentials, cart context. Adds purchase protection if agent errs</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>N/A (infra; tokens spent on partner platforms)</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>Apr-2026</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>S17</t>
         </is>
@@ -2637,30 +3053,40 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
+          <t>Front-end (merchants reachable from ChatGPT/Copilot/etc.)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
           <t>OpenAI ACP, Google UCP, Agent Payments Protocol</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>OpenAI, Google, Perplexity, Microsoft Copilot, Wix, Cymbio, Shopware</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Live Oct-2025</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>MCP servers since Apr-2025; gives PP merchants instant agentic acceptance with fraud + buyer protection</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Low (MCP server traffic; tokens external)</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>Oct-2025</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>S18</t>
         </is>
@@ -2684,30 +3110,40 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
+          <t>Front-end (rails for external agents like ChatGPT)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
           <t>Agentic Commerce Protocol (ACP); MPP</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>OpenAI (co-author of ACP), URBN, Etsy, Coach, Kate Spade, Wix, BigCommerce</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Beta 2025-2026</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Shared Payment Tokens reduce fraud; modular product discovery + checkout APIs</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>N/A (infra)</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>2025 (beta); 2026 GA in progress</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>S19</t>
         </is>
@@ -2731,30 +3167,40 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
+          <t>Front-end (acceptance for AI agents)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
           <t>Mastercard Agent Pay framework; Visa Trusted Agent Protocol</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Mastercard, Visa</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Live Mar-2026</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Routes AI-initiated transactions through standard card-processing infrastructure</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>N/A (infra)</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Mar-2026</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>S20</t>
         </is>
@@ -2778,30 +3224,40 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
+          <t>Front-end (merchant-facing) + Back-end (merchant guardrails)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
           <t>Google UCP, AP2, Visa Trusted Agent Protocol</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Google, Visa; Agentic AI Foundation member</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Live (joined foundation Dec-2025)</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Tokenisation cost claimed -30%; framework keeps merchants in control of relationship/data</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>N/A (infra) + Low for control-framework reasoning</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>Dec-2025 → 2026</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>S21</t>
         </is>
@@ -2825,30 +3281,40 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
+          <t>Back-end (issuer enablement) + Front-end (auth flows)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
           <t>Visa Trusted Agent Protocol, Mastercard Agent Pay</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Mastercard, Visa</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>GA end Q1-2026</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Adds KYA + agent-aware authorisation, fraud, dispute frameworks for issuing banks</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>N/A (infra)</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>Jan-2026</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>S22</t>
         </is>
@@ -2872,30 +3338,40 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
+          <t>Front-end (consumer-facing marketplace agent)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
           <t>Multi-protocol; partners with Visa, Mastercard, Google</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Visa, Mastercard, Google, top retailers</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Pilot</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Redesigning loyalty &amp; financing to be AI-readable; running own marketplace agent</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Low (pilot scale)</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>S23</t>
         </is>
@@ -2919,30 +3395,40 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
+          <t>Both (potential)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
           <t>Industry protocols (early integration)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>n/a public</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Exploration</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Bernstein names Block among fintechs positioned for agentic-commerce upside; specific shipping product not yet public</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>S24</t>
         </is>
@@ -2959,17 +3445,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="48" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="43" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2995,20 +3483,30 @@
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
+          <t>Role (Front-end / Back-end)</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
           <t>Underlying tech / partners</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Stage (2026)</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Adoption / Impact</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Token consumption (tier)</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Source ID</t>
         </is>
@@ -3037,20 +3535,30 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>Front-end</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>In production but partial reversal in 2026</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>2.3M chats/month at peak (~700 FTE equivalent); resolution 11→2 min; targeted ~$40M profit lift in 2024. Partial human re-hiring announced 2026 after CSAT slipped</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Very High (28M+ chats/yr)</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>S25</t>
         </is>
@@ -3079,20 +3587,30 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
+          <t>Both (call-centre co-pilot back-end; consumer assistant front-end)</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>In production</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Resolves 55% of L1 queries; chat response time -70%; covers 5,000+ employees and 114M+ customers</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Very High (114M+ customers)</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>S26</t>
         </is>
@@ -3121,20 +3639,30 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
+          <t>Front-end</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
           <t>Internal + partners (zero-retention 3rd party)</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Launched Apr-2026</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>13M UK customers in scope; biometric approval for sensitive actions</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Very High (13M UK customers; multimodal)</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>S26</t>
         </is>
@@ -3163,20 +3691,30 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
+          <t>Front-end</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
           <t>Internal</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Launched Mar-2026</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>First UK agentic financial assistant per coverage; handles savings goals, bill organisation</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>S26</t>
         </is>
@@ -3205,20 +3743,30 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
+          <t>Front-end</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
           <t>Internal + partners</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Used for support and personalisation across consumer base</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>S26</t>
         </is>
@@ -3247,20 +3795,30 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
+          <t>Both (employee-facing in customer companies; back-end in Brex)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
           <t>Internal + Anthropic Claude</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Auto-approves low-risk expenses; categorises violations; eliminates expense busywork</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>High (per-transaction reasoning at scale)</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>S27</t>
         </is>
@@ -3289,20 +3847,30 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
+          <t>Back-end (finance ops) + Front-end touch (employee chat)</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
           <t>Internal AI</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>99% OCR accuracy; 2.4x faster invoice processing; 7x fewer clicks per bill</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>S27</t>
         </is>
@@ -3331,20 +3899,30 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
           <t>Internal</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Live; raised $100M Series C at $1.4B (2026)</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Ribbit, Khosla, Goodwater led round; positioned as 'autonomous finance function'</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>S28</t>
         </is>
@@ -3373,20 +3951,30 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
+          <t>Back-end (mostly)</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
           <t>Internal + partners</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Less public agentic detail than peers; focus on AI-assisted UX</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Low / N/D</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>S27</t>
         </is>
@@ -3403,16 +3991,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="46" customWidth="1" min="3" max="3"/>
     <col width="41" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="46" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="47" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3438,15 +4028,25 @@
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
+          <t>Role (Front-end / Back-end)</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
           <t>Notable customers / proof points</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Stage / Funding</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Token consumption (tier)</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Source ID</t>
         </is>
@@ -3475,15 +4075,25 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>Back-end (analyst-facing)</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>Serves clients with $30T AUM; 1.5B pages processed; ~200k prompts/day</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Raised ~$161M; mid/high six-figure ACVs</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Very High (long-context document agents)</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
@@ -3512,15 +4122,25 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
+          <t>Back-end</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
           <t>Used in financial services among 1000+ customers</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Raised ~$765M (Series F)</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
@@ -3549,15 +4169,25 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
+          <t>Back-end</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
           <t>Used by leading law firms; expanding into FS</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Multi-billion valuation per public reporting</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
@@ -3586,15 +4216,25 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
+          <t>Both (model layer for either)</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
           <t>RBC co-developed 'North for Banking'</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Late-stage scale-up</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Very High (foundation model provider)</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>S13</t>
         </is>
@@ -3623,15 +4263,25 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
+          <t>Back-end</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
           <t>Up to 18,300 analyst hrs/yr saved; 95% of screening hits auto-resolved; 50% lower doc processing time</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Established vendor</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>S30</t>
         </is>
@@ -3660,15 +4310,25 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
+          <t>Back-end</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
           <t>70% reduction in EDD queue completion; $5.35M first-year ops savings; 200k+ customer reviews automated</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Startup</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>S30</t>
         </is>
@@ -3697,15 +4357,25 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
+          <t>Back-end</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
           <t>Used by fintech startups for audit-ready compliance</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Startup</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>S30</t>
         </is>
@@ -3734,15 +4404,25 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
+          <t>Back-end</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
           <t>Reduces false positives in watchlist screening; mimics human reviewer</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Public-co vendor</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>S22</t>
         </is>
@@ -3771,15 +4451,25 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
           <t>Up to 70% manual workload cut; 65% AML investigation time cut at one client</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Raised $50M Series A 2026</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>S28</t>
         </is>
@@ -3808,15 +4498,25 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
+          <t>Back-end</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
           <t>30+ enterprise customers; 100k hours saved/year</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Raised $23M Series A (Lightspeed) 2026</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>S28</t>
         </is>
@@ -3845,15 +4545,25 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
+          <t>Back-end</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
           <t>Addresses analyst staffing shortages</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Raised $15M 2026</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>S28</t>
         </is>
@@ -3882,15 +4592,25 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
+          <t>Front-end (rails consumed by external agents)</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
           <t>Pre-seed product; payments layer for safe agent workflows</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Raised £1.8M pre-seed 2026</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>N/A (infra)</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>S28</t>
         </is>
@@ -3919,15 +4639,25 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
+          <t>Back-end</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
           <t>Built on NVIDIA AI Factory + KX time-series DB; launched at GTC 2026</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Public-co vendor</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>S31</t>
         </is>
@@ -3956,15 +4686,25 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
+          <t>Back-end</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
           <t>Goldman Sachs deployed across 12k engineers</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Late-stage startup</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Very High (long-horizon coding agent)</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>S4</t>
         </is>
@@ -3993,15 +4733,25 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
+          <t>Front-end (rails consumed by external agents)</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
           <t>Competes with x402; agent-pay rails</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Startup</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>N/A (infra)</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>S32</t>
         </is>
@@ -4030,15 +4780,25 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
+          <t>Front-end (rails consumed by external agents)</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
           <t>Tracks ACP, AP2, MPP, x402 protocol landscape</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Startup</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>N/A (infra)</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>S32</t>
         </is>

</xml_diff>

<commit_message>
Add coding-vs-FS contrast and leading-companies sheets
Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/agentic_ai_banking_payments.xlsx
+++ b/data/agentic_ai_banking_payments.xlsx
@@ -15,7 +15,9 @@
     <sheet name="5_Enterprise_Platforms" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="6_Agentic_Payments_Protocols" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="7_Funding_Rounds" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="8_Sources" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="8_Coding_vs_FS_Contrast" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="9_Leading_Companies" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="10_Sources" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -444,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -649,12 +651,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>8_Sources</t>
+          <t>8_Coding_vs_FS_Contrast</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>URLs and publications used to compile this tracker.</t>
+          <t>Side-by-side: how coding agents differ from banking, payments and FS agents on tokens / task duration / cost / reliability.</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -664,109 +666,2372 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n"/>
-      <c r="B16" s="2" t="n"/>
-      <c r="C16" s="2" t="n"/>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>9_Leading_Companies</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Pick of the leader(s) in each agent category.</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>see sheet</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>10_Sources</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>URLs and publications used to compile this tracker.</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>see sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n"/>
+      <c r="B18" s="2" t="n"/>
+      <c r="C18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
           <t>Definitions</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n"/>
-      <c r="C17" s="2" t="n"/>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Agentic AI</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>AI systems that plan and execute multi-step tasks across tools and data, with limited human prompting (vs. single-turn chat or copilot).</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Agentic commerce</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Purchases initiated by an AI agent on behalf of a consumer or business, using tokenised credentials and intent attestations.</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>KYA</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Know-Your-Agent — analogue of KYC where the network/issuer authenticates the AI agent itself.</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Role: Front-end</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Agent interacts directly with external counterparties — retail or wholesale customers, merchants, dealers, or third-party AI surfaces (e.g., ChatGPT). Drives revenue, CX or distribution.</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Role: Back-end</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Agent runs inside the institution — employee productivity, ops, compliance, software engineering, treasury, finance, risk. Drives cost, throughput or control.</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Role: Both</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Same product line spans customer-facing and internal-facing surfaces (e.g., a contact-centre platform that powers both bot self-service and agent assist).</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Token consumption tiers</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Qualitative monthly token-usage estimate based on scale (users × interactions × avg tokens). Buckets: Very High (&gt;1B tokens/mo), High (100M–1B), Medium (10M–100M), Low (&lt;10M), N/A (not LLM-based or pure infra), N/D (not disclosed). Estimates are illustrative — vendors rarely publish exact figures.</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Sub-category</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Leader</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Why leader</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Source ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Coding agents</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Autonomous SWE (long-horizon)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Cognition (Devin)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>First major-bank-scale deployment (Goldman Sachs, 12k engineers); ACU-based pricing; 67% PR merge rate; 25h-class runs documented elsewhere in category.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>S4, S40</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Coding agents</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>IDE-embedded coding agent</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Cursor</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>$2k–$5k/team/month observed agent spend; Sonnet ~$0.09/request default; widely adopted by banks' engineering orgs.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>S41</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Coding agents</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Coding agent CLI / inline</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic (Claude Code)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Long-context, cache-optimised sessions; the de-facto choice for long-horizon back-end runs at finance customers (Brex, Coinbase, Citi via Claude FS).</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>S20, S39</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Coding agents</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Cloud SWE agent (asynchronous)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI (Codex)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>GA pricing on gpt-5.2-codex; documented 25h / 13M-token long-horizon runs; native to ChatGPT Enterprise stack used at BBVA, Santander, NatWest.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>S42</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Coding agents</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>DevOps / git platform agent</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>GitHub (Copilot agent mode + Workspace)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Most widely distributed coding agent (Free→Enterprise tiers); 1M+ token Workspace context; embedded in Microsoft FS stack.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>S43</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Coding agents</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Frontier-model autonomy benchmark leader</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic Claude Opus 4.6</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>~14.5h on METR Time-Horizon 1.1 (50% reliability) – longest sustained autonomy in early 2026.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>S38</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Banking — incumbent rollout</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise productivity at scale</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase (LLM Suite + 450+ agentic use cases)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>230k–250k seat reach; targets 1,000 production agents; 3–6 hr/wk per-user productivity claim; backed by $18B tech budget.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Banking — incumbent rollout</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Investment banking agentic ops</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Goldman Sachs (Claude Opus + Devin + GS AI Assistant)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Most aggressive front-to-back agentic deployment among bulge brackets: trade accounting, compliance, surveillance, IB pitchbooks, 12k engineers on Devin.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>S4, S20</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Banking — incumbent rollout</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Consumer agentic banking</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Wells Fargo (Fargo + Agentspace) and Bank of America (Erica)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Wells: 215k employees + Gemini-Enterprise consumer agents. BofA: 42M consumer users, ~11k FTE-equivalent throughput.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>S2, S6</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Banking — incumbent rollout</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Wealth management</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Morgan Stanley (AI @ MS Assistant + Debrief)</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>98% advisor-team adoption; ~15k advisors; 1M Zoom calls/yr automated; reference for OpenAI in FS.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>S5</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Banking — Europe</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Most aggressive agentic rollout</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>ING Bank (agentic mortgage origination + voice agents)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Live agentic mortgages (NL, DE) targeted 2026; €350M cost savings, 1,250 ops job exits projected.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>S11</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Banking — Europe</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Largest enterprise OpenAI deployment</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>BBVA (ChatGPT Enterprise to 120k staff)</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>10x scale-up in 2025; 20k+ custom GPTs; 83% weekly active in pilot; pairs with Blue customer assistant.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Banking — Asia/EM</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Production-grade agentic bank</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>DBS Bank (DBS Joy + CodeBuddy)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>S$1B AI-driven economic value FY25; agentic governance via PURE framework.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Banking — Canada</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Agentic strategy leader</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Royal Bank of Canada (RBC AI Group + Cohere 'North for Banking')</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Dedicated AI Group reporting to CEO; targets up to C$1B value by 2027; #3 globally for FS AI maturity per coverage.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Payments — networks</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Agentic commerce platform leader</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Visa (Intelligent Commerce Connect)</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Apr-2026 launch; supports four protocols (Visa TAP, MPP, ACP, UCP); positioned as neutral payment rail for agents.</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>S16</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Payments — networks</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Agentic commerce framework leader</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Mastercard (Agent Suite, Agent Pay, Verifiable Intent)</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Q2-2026 launch; cryptographic dispute trail; integrated with Fiserv US merchant base.</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>S16</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Agentic AI</t>
+          <t>Payments — issuers</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>AI systems that plan and execute multi-step tasks across tools and data, with limited human prompting (vs. single-turn chat or copilot).</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="n"/>
+          <t>Agentic issuer SDK</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>American Express (ACE developer kit + Agent Purchase Protection)</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Apr-2026 launch; first issuer to add explicit purchase protection for agent errors.</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>S17</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Agentic commerce</t>
+          <t>Payments — wallets / acceptance</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Purchases initiated by an AI agent on behalf of a consumer or business, using tokenised credentials and intent attestations.</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="n"/>
+          <t>Agentic checkout reach</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>PayPal (Agent Ready + Store Sync)</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Live Oct-2025; instantly enables tens of millions of merchants across OpenAI, Google, Microsoft Copilot, Perplexity.</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>S18</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>KYA</t>
+          <t>Payments — acquiring infra</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Know-Your-Agent — analogue of KYC where the network/issuer authenticates the AI agent itself.</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="n"/>
+          <t>Open agentic checkout protocol</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Stripe (Agentic Commerce Suite + ACP with OpenAI)</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Co-author of ACP; powers ChatGPT Instant Checkout; Shared Payment Tokens reduce fraud.</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Role: Front-end</t>
+          <t>Payments — processors</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Agent interacts directly with external counterparties — retail or wholesale customers, merchants, dealers, or third-party AI surfaces (e.g., ChatGPT). Drives revenue, CX or distribution.</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="n"/>
+          <t>Agentic merchant processing</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Fiserv</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Routes Mastercard Agent Pay through millions of US merchants; also integrated with Visa Trusted Agent Protocol.</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>S20</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Role: Back-end</t>
+          <t>Payments — issuing tech</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Agent runs inside the institution — employee productivity, ops, compliance, software engineering, treasury, finance, risk. Drives cost, throughput or control.</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="n"/>
+          <t>Agentic core for banks</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>FIS (agentic commerce issuing platform)</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>First issuer-side enablement: KYA + agent-aware auth, fraud, dispute frameworks; partnered with Visa + Mastercard.</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>S22</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Role: Both</t>
+          <t>FS — neobanks / fintech</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Same product line spans customer-facing and internal-facing surfaces (e.g., a contact-centre platform that powers both bot self-service and agent assist).</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="n"/>
+          <t>Agentic consumer assistant</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Revolut (AIR)</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Apr-2026 launch to 13M UK customers; spending, investing, subscriptions, card controls, travel — single multimodal agent.</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>S26</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Token consumption tiers</t>
+          <t>FS — neobanks / fintech</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Qualitative monthly token-usage estimate based on scale (users × interactions × avg tokens). Buckets: Very High (&gt;1B tokens/mo), High (100M–1B), Medium (10M–100M), Low (&lt;10M), N/A (not LLM-based or pure infra), N/D (not disclosed). Estimates are illustrative — vendors rarely publish exact figures.</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="n"/>
+          <t>Agentic customer service at scale</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Klarna + Nubank (OpenAI)</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Klarna: 700-FTE-equivalent at peak, even after 2026 partial reversal. Nubank: 55% L1 resolution, -70% chat response time, covers 114M+ customers.</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>S25, S26</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>FS — neobanks / fintech</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Agentic finance ops (B2B)</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Brex + Ramp</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Brex: Anthropic-powered expense / audit agents. Ramp: 99% OCR, 2.4x faster invoice processing, agentic AP.</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>S27</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>FS — vendors</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Finance research agents</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Hebbia</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Clients with $30T AUM; 1.5B pages processed; ~200k prompts/day; deepest finance-specific agent library.</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>FS — vendors</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Compliance / financial-crime agents</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Fenergo (FinCrime OS) + Bretton</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Fenergo: 95% of screening hits auto-resolved, up to 18.3k analyst hrs/yr saved. Bretton: 70% EDD queue cut, $5.35M first-year savings.</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>S30</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>FS — vendors</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Capital-markets agentic blueprint</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>KX (with NVIDIA)</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Two GTC-2026 blueprints: Research Assistant + Trading Signal Agent on NVIDIA AI Factory + KX time-series DB.</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>S31</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>FS — platforms</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Foundation model for FS agents (US/Europe)</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Backbone for BBVA, Santander, NatWest assistant, Klarna, Nubank, Morgan Stanley; co-author of ACP for agentic commerce.</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>S36</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>FS — platforms</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Foundation model for back-office FS agents</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic (Claude for Financial Services)</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Goldman Sachs core ops, Citi, Brex, Coinbase; Claude for Excel; finance-specific connectors (S&amp;P, FactSet, Morningstar, LSEG).</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>S20</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>FS — platforms</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Hyperscaler enterprise agentic platform</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Google Cloud (Gemini Enterprise / Agentspace)</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Bank-wide rollouts: Wells Fargo (215k staff), HSBC selected workloads; powers Citi Stylus alongside Anthropic.</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>S34</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>FS — platforms</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>CRM-anchored agentic platform</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Salesforce (Agentforce for Financial Services)</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Pre-built advisor / banker / service / collections agents; Atlas Reasoning Engine; large FS install base.</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>S37</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Coding-agent infra</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Frontier coding model</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic Claude (Sonnet/Opus) — chosen by Cursor, Claude Code, Brex, Goldman Sachs</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Default model for highest-reliability coding sessions; longest METR autonomy horizon at Opus 4.6.</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>S20, S38, S39</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Agentic-payments protocols</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Open consumer-checkout standard</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Agentic Commerce Protocol (OpenAI + Stripe)</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Powers ChatGPT Instant Checkout; adopted by Etsy, Shopify (1M+ merchants), URBN, Coach, Kate Spade, PayPal MCP server.</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>S36</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Agentic-payments protocols</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Network-rail standard</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Visa Trusted Agent Protocol</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Live in Visa ICC; supported by AWS, Aldar, Firmly, Nekuda, Fiserv, Adyen.</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>S16</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Agentic-payments protocols</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Crypto / stablecoin native</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>x402 (Coinbase + Linux Foundation)</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Apr-2026 launch; sub-cent micropayments in stablecoins; backed by Stripe, Cloudflare, AWS, Google, Microsoft, Visa, Mastercard via X402 Foundation.</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>S32</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Source ID</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Publisher</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Accessed</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>CeFPro / The Digital Banker / aibmag.com / emerj</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>JPMorgan LLM Suite &amp; agentic AI rollout coverage</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>https://connect.cefpro.com/article/view/inside-jpmorgan-llm-suite-as-ai-agents-spread-across-the-bank</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>American Banker / Fortune / BofA Newsroom / CIO</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Bank of America Erica + AskGPS coverage</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>https://newsroom.bankofamerica.com/content/newsroom/press-releases/2025/09/bofa-s-new-genai-assistant-transforms-global-payments-solutions.html</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Citi / FinancialIT / The Register / pymnts / CIO Dive</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Citi Stylus Workspaces with agentic AI</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.citigroup.com/global/news/press-release/2025/citi-unveils-citi-stylus-workspaces-agentic-ai-turbocharging-productivity</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Economic Times / FinancialContent / Bankers' Magazine / Observer</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Goldman Sachs GS AI Assistant, Devin, Anthropic deployment</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>https://m.economictimes.com/tech/artificial-intelligence/goldman-sachs-launches-ai-assistant-firmwide-memo-shows/articleshow/122031424.cms</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>S5</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Morgan Stanley / OpenAI / Nasdaq / CNBC</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>AI @ Morgan Stanley Assistant + Debrief</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.morganstanley.com/press-releases/ai-at-morgan-stanley-debrief-launch</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Wells Fargo / Google Cloud / National Mortgage News / American Banker</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Wells Fargo Fargo + Agentspace deployment</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/blog/topics/financial-services/wells-fargo-agentic-ai-agentspace-empowering-workers</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>S7</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Stack-ai / Barclays Private Bank / Barclays.com</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>HSBC and Barclays agentic AI deployment notes</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>https://privatebank.barclays.com/insights/ai-outlook-2026-11-2025/agentic-ai-a-little-less-conversation-a-little-more-action-pleas/</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>S8</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>UBS / Yahoo Finance / Stack-ai</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>UBS &amp; Deutsche Bank agentic AI strategy</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ubs.com/global/en/careers/about-us/stories/2025/agentic-ai.html</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>S9</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>The Asian Banker / FStech / National Technology</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Lloyds, NatWest, Santander agentic AI plans 2026</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theasianbanker.com/press-releases/lloyds-scales-genai-and-agentic-ai-targets-127m-in-value-creation-for-2026</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI / opentools.ai</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>BBVA + OpenAI ChatGPT Enterprise rollout</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>https://openai.com/index/bbva-collaboration-expansion/</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Computer Weekly / FStech / Dutch IT Leaders</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>ING agentic AI mortgages and voice agents</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.computerweekly.com/news/366626743/ING-Bank-transforming-operations-through-agentic-AI</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>DBS / Computer Weekly / Business Times / Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>DBS Bank agentic AI (DBS Joy, CodeBuddy)</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dbs.com/artificial-intelligence-machine-learning/artificial-intelligence/agentic-ai-is-here-are-we-ready-to-govern-it.html</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Cedar Report / Newswire / Fintech.ca / RBCCM</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Canadian banks agentic AI (RBC, TD, Scotia, BMO, CIBC)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cedarreport.com/guides/how-canadian-banks-are-using-ai-in-2026-rbc-td-bmo-and-more</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>S14</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>The Financial Brand / Capital One / TechCrunch / NVIDIA On-Demand</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Capital One Chat Concierge + agentic AI</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>https://thefinancialbrand.com/news/banking-products/capital-ones-chat-concierge-puts-agentic-ai-on-car-dealers-websites-187128</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>S15</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Truist IR / PNC / American Banker / FinancialContent</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Truist receivables, PNC working capital, US Bank developer assistant</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>https://ir.truist.com/2026-02-03-Truist-launches-AI-enabled-receivables-platform-to-accelerate-cash-application-and-minimize-exceptions</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>S16</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>TheLetterTwo / Digital Commerce 360 / American Banker / ClearingPost / adwaitx</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Visa Intelligent Commerce Connect, Mastercard Agent Suite/Pay</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>https://thelettertwo.com/2026/04/08/visa-wants-to-be-the-payment-rail-for-the-agentic-economy</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>S17</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Digital Commerce 360 / Fortune</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>American Express ACE developer kit + Agent Purchase Protection</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.digitalcommerce360.com/2026/04/14/american-express-agentic-commerce-developer-kit-purchase-protection/</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>S18</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>PayPal Newsroom / PayPal Tech Blog / PayPal.ai</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>PayPal Agent Ready, Store Sync, MCP servers</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>https://newsroom.paypal-corp.com/2025-10-28-PayPal-Launches-Agentic-Commerce-Services-to-Power-AI-Driven-Shopping</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Stripe blog / Stripe docs / agenticcommerce.expert / GitHub</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Stripe Agentic Commerce Suite + ACP</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>http://www.stripe.com/blog/agentic-commerce-suite</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>S20</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic / Economic Times / ETCFO / ClaudeReadiness</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Claude for Financial Services + Goldman Sachs deployment</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.anthropic.com/solutions/financial-services</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>S21</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Adyen / Major Matters</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Adyen agentic-commerce strategy + Universal Token Vault</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adyen.com/knowledge-hub/adyen-joins-agentic-ai-foundation</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>S22</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>FIS press / Temenos</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>FIS agentic commerce platform + Temenos FCM AI Agent</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fisglobal.com/about-us/media-room/press-release/2026/fis-launches-industry-first-ai-transaction-platform-to-help-banks-lead</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>S23</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Synchrony Newsroom</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Synchrony agentic-commerce strategy</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.synchrony.com/contenthub/insights/blog-post-by-mike-storiale.html</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>S24</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Markets Insider (Bernstein note)</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Bernstein bullish on Fiserv, Block, Adyen for agentic commerce</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>https://markets.businessinsider.com/news/stocks/fiserv-block-and-adyen-here-s-why-bernstein-is-bullish-on-these-3-fintech-stocks-1035185068</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>S25</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI / ad-hoc-news / myaskai / Klarna</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Klarna AI assistant plus 2026 reversal coverage</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ad-hoc-news.de/boerse/news/ueberblick/klarna-s-ai-pivot-reversing-course-after-customer-service-setbacks/69026000</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>S26</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>FStech / FinTech Weekly / Marcel van Oost / Fintyle</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Nubank, Revolut AIR, Starling Assistant, Monzo coverage</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fintechweekly.com/news/revolut-air-ai-assistant-uk-customers-launch-2026</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>S27</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Brex.ai / Ramp blog / Stack-ai</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Brex Agents + Ramp agentic AP and expense</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.brex.ai/</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>S28</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>SiliconANGLE / aihaberleri / theoutpost / stacks.ai / uktech.news</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>2026 agentic-AI fintech funding rounds (Slash, Dyna.Ai, Stacks, EnFi, Ralio)</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>https://siliconangle.com/2026/04/16/slash-raises-100m-1-4b-valuation-expand-ai-powered-banking-platform-online-businesses/</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Hebbia / V7Labs / CB Insights</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Hebbia, Glean, Harvey product + funding profiles</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hebbia.com/blog/whats-new-april-disclosure-2026</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>S30</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Fenergo / Bretton / Stack-ai / dev.to</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Compliance / financial-crime agentic vendors</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>https://fenergo.com/agentic-ai-agents</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>S31</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>KX / NVIDIA On-Demand / NVIDIA blog</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>KX agentic AI blueprints + Capital One GTC 2026 talk + NVIDIA FS survey</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>https://kx.com/news-room/kx-launches-agentic-ai-blueprints-powered-by-nvidia-at-gtc-2026-featuring-a-capital-markets-research-assistant-and-trading-signal-agent/</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>S32</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Coinbase / Linux Foundation / Crossmint / aiagentstore</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>x402 protocol launch + Skyfire / Crossmint comparison</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>https://blog.crossmint.com/what-is-x402/</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>S33</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft Learn / Microsoft Industry Blog / myabt / Microsoft Adoption</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft Finance Agents + Agent 365 + Copilot for FS</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.microsoft.com/en-us/industry/blog/financial-services/banking/2026/02/26/the-agentic-moment-in-banking-a-blueprint-for-better-customer-experiences/</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>S34</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Google Cloud / Promevo / ScaleByTech</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Gemini Enterprise (Agentspace) for banking</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/agentspace</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>S35</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Google / Adyen / Crossmint</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Universal Commerce Protocol (UCP) + Agent Payments Protocol (AP2)</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.crossmint.com/learn/agentic-payments-protocols-compared</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>S36</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI / OpenAI Developers / Ekamoira</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>ChatGPT Instant Checkout + Agentic Commerce Protocol</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>https://openai.com/index/buy-it-in-chatgpt/</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>S37</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Salesforce / Vantage Point</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Agentforce for Financial Services</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.salesforce.com/financial-services/artificial-intelligence/</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>S38</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>METR (Model Evaluation &amp; Threat Research)</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Time-horizon benchmark for frontier coding agents (v1.1, Jan-2026)</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>https://metr.org/time-horizons</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>S39</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>TokenCost / Anthropic GitHub issues</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Claude Code per-session token economics (cache, regressions)</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>https://tokencost.app/blog/claude-code-cost-per-session</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>S40</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Devin docs / vibecoder.me / imseankim.com</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Devin ACU pricing, SWE-bench performance, cost per task</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>https://docs.devin.ai/admin/billing</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>S41</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Cursor docs / AgentCost / Cursor blog</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Cursor agent request pricing and team usage patterns</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>https://cursor.com/docs/account/teams/pricing</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>S42</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI Codex docs / Hypereal AI / TokenCost</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Codex token consumption per task; long-horizon 25h / 13M-token run</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>https://developers.openai.com/codex/cookbook/long_horizon_tasks/</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>S43</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>GitHub Docs / GitHub features</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>GitHub Copilot agent-mode / premium-request pricing 2026</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>https://docs.github.com/en/billing/concepts/product-billing/github-copilot-premium-requests</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>S44</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Otera / Medium (S. Boddula) / blogarama / paxrel</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Banking AI agent task durations: KYC in 8s, onboarding in minutes vs days</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>https://www.otera.ai/solutions/banking-autonomous-kyc-and-onboarding</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5905,1039 +8170,283 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="37" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
+          <t>Dimension</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Coding agents</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Banking / Payments / FS agents</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Why the gap</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
           <t>Source ID</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>Publisher</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>Accessed</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>Primary task type</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>CeFPro / The Digital Banker / aibmag.com / emerj</t>
+          <t>Open-ended software engineering: write/refactor code, run tests, ship PRs, debug, ops scripting, autonomous research.</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>JPMorgan LLM Suite &amp; agentic AI rollout coverage</t>
+          <t>Bounded transactional workflows: customer Q&amp;A, KYC/AML, fraud triage, treasury actions, IB document drafting, payments auth.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>https://connect.cefpro.com/article/view/inside-jpmorgan-llm-suite-as-ai-agents-spread-across-the-bank</t>
+          <t>Code is unbounded, exploratory and stateful; banking work is regulated, schema-heavy and must be auditable.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>S38, S40, S42, S44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>Typical task duration</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>American Banker / Fortune / BofA Newsroom / CIO</t>
+          <t>Minutes to many hours per task. SWE-bench / live work: 1–30 min average; complex refactors half-day; documented Codex run was 25 hours / 30k LOC. METR Time-Horizon 1.1 (Jan-2026) shows Opus 4.6 ≈14.5h, GPT-5.2 ≈6.6h, Opus 4.5 ≈4.8h at 50% reliability; horizon doubling ~every 4 months.</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Bank of America Erica + AskGPS coverage</t>
+          <t>Seconds to a few minutes per autonomous task: KYC decisions in ~8s, edge-case review ~2 min, onboarding compressed from 24+ days to 'minutes', call-centre answers &lt;30s. Multi-step IB / compliance workflows can run minutes to low single-digit hours.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>https://newsroom.bankofamerica.com/content/newsroom/press-releases/2025/09/bofa-s-new-genai-assistant-transforms-global-payments-solutions.html</t>
+          <t>Coding is long-horizon planning + tool use; FS work is mostly short, tightly-scoped retrieval/decision turns under SLAs and human-in-loop policy.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>S38, S42, S44</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>S3</t>
+          <t>Median tokens per task</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Citi / FinancialIT / The Register / pymnts / CIO Dive</t>
+          <t>Simple bug fix: ~20–35k total. Medium feature: ~120–140k. Half-day refactor: ~500–600k. Multi-agent run: 1.5M+ (Haiku/Sonnet mix). Codex long-horizon documented run: ~13M tokens.</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Citi Stylus Workspaces with agentic AI</t>
+          <t>Self-service chat turn: low thousands of tokens. Agentic workflow turn (KYC, fraud, IB pitch slide): tens of thousands. End-to-end compliance case: ~100k–300k. Rare multi-agent research run reaches low millions.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>https://www.citigroup.com/global/news/press-release/2025/citi-unveils-citi-stylus-workspaces-agentic-ai-turbocharging-productivity</t>
+          <t>Coding agents iterate on full repos with long context; FS agents stitch short structured retrievals + policy checks.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>S39, S40, S42, S44</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>Cost per task (list price)</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Economic Times / FinancialContent / Bankers' Magazine / Observer</t>
+          <t>Claude Code: $0.07–$3 per typical session; multi-agent runs $3–$7+. Devin ACUs ~$2.25 each; complex tasks $3–$15. Cursor Sonnet ~$0.09/request; heavy refactor session ~$20. Codex small task ~$0.16; medium ~$1–$3.</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Goldman Sachs GS AI Assistant, Devin, Anthropic deployment</t>
+          <t>Per-conversation cost generally well under $1; even Salesforce Agentforce lists $2/conversation or $0.10/action. Compliance vendors price per case (e.g., Fenergo claims 95% screening hits auto-resolved at low marginal cost).</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>https://m.economictimes.com/tech/artificial-intelligence/goldman-sachs-launches-ai-assistant-firmwide-memo-shows/articleshow/122031424.cms</t>
+          <t>Coding tasks burn long, exploratory contexts; FS tasks reuse templated prompts + RAG hits.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>S37, S39, S40, S41, S42</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>S5</t>
+          <t>Tokens / month, leading deployments</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Morgan Stanley / OpenAI / Nasdaq / CNBC</t>
+          <t>Per-engineer: a daily Claude Code user can spend $20–$100/day → tens of millions of tokens/day; Goldman's 12k Devin seats and any 10k+ engineer Copilot/Cursor base imply &gt;&gt;10B tokens/month at the firm level.</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>AI @ Morgan Stanley Assistant + Debrief</t>
+          <t>Per-customer: a BBVA / Santander seat is hundreds of thousands–low millions tokens/month; consumer chat (Erica, Klarna, Nubank, Revolut AIR) at tens of millions of users still aggregates into multi-billion tokens/month, but with much smaller per-event tokens.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>https://www.morganstanley.com/press-releases/ai-at-morgan-stanley-debrief-launch</t>
+          <t>Coding = few users × very heavy per-user usage. FS = many users × light per-user usage. Both can land at 'Very High' tier but via different shapes.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>S39, S40, S41, S42</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>S6</t>
+          <t>Reliability requirement</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Wells Fargo / Google Cloud / National Mortgage News / American Banker</t>
+          <t>Tolerant of failure: PRs reviewed by humans; failed runs are cheap to retry. Benchmarks reported at 50% / 80% reliability.</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Wells Fargo Fargo + Agentspace deployment</t>
+          <t>Strict: regulated decisions (KYC, lending, payment auth) need explainability, audit, low false-positive rates. Frameworks like Barclays / HSBC 'tiered autonomy', DBS PURE, NatWest human-in-loop.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>https://cloud.google.com/blog/topics/financial-services/wells-fargo-agentic-ai-agentspace-empowering-workers</t>
+          <t>Asymmetric cost of error: a wrong code change is reversible; a wrong AML decision is a regulatory event.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>S7, S12, S30, S44</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>S7</t>
+          <t>Tool surface</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Stack-ai / Barclays Private Bank / Barclays.com</t>
+          <t>IDE + shell + browser + git + cloud: very wide tool-use surface, often dozens of tools per session.</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>HSBC and Barclays agentic AI deployment notes</t>
+          <t>Closed enterprise stack: core banking, CRM (Salesforce), data warehouse, screening DBs, ERP. Mediated by MCP / Agent 365 / Agentforce / Agentspace.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>https://privatebank.barclays.com/insights/ai-outlook-2026-11-2025/agentic-ai-a-little-less-conversation-a-little-more-action-pleas/</t>
+          <t>Coding agents need general-purpose tool use; FS agents need governed connectors with RBAC and DLP.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>S33, S34, S37</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>S8</t>
+          <t>Pricing / monetisation model</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>UBS / Yahoo Finance / Stack-ai</t>
+          <t>Per-seat unlimited (Copilot $10–$39/mo) increasingly replaced by usage-based ACU / token / request pricing (Devin, Cursor, Codex API).</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>UBS &amp; Deutsche Bank agentic AI strategy</t>
+          <t>Mostly bundled into enterprise contracts with the bank's platform vendor (Salesforce, Microsoft, Google, Anthropic, OpenAI). Some action-based pricing emerging (Agentforce $0.10/action, $2/conversation).</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>https://www.ubs.com/global/en/careers/about-us/stories/2025/agentic-ai.html</t>
+          <t>Coding usage is metered because elastic; FS usage is negotiated because procurement-led and capacity-planned.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>S37, S40, S41, S42, S43</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>S9</t>
+          <t>Front-end vs back-end mix</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>The Asian Banker / FStech / National Technology</t>
+          <t>Almost entirely back-end (developer-facing). Devin, Codex, Cursor, Claude Code, Copilot all run inside the engineering org.</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Lloyds, NatWest, Santander agentic AI plans 2026</t>
+          <t>Roughly balanced: Front-end (Erica, Fargo, Cora, AIR, Klarna, Nubank, Capital One Chat Concierge, network rails) plus heavy Back-end (LLM Suite, GS Claude ops, Stylus, Hebbia, Fenergo).</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>https://www.theasianbanker.com/press-releases/lloyds-scales-genai-and-agentic-ai-targets-127m-in-value-creation-for-2026</t>
+          <t>Coding is an internal productivity vector; FS spans CX, distribution and ops.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>S10</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>OpenAI / opentools.ai</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>BBVA + OpenAI ChatGPT Enterprise rollout</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>https://openai.com/index/bbva-collaboration-expansion/</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>S11</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Computer Weekly / FStech / Dutch IT Leaders</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>ING agentic AI mortgages and voice agents</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.computerweekly.com/news/366626743/ING-Bank-transforming-operations-through-agentic-AI</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>S12</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>DBS / Computer Weekly / Business Times / Yahoo Finance</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>DBS Bank agentic AI (DBS Joy, CodeBuddy)</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>https://www.dbs.com/artificial-intelligence-machine-learning/artificial-intelligence/agentic-ai-is-here-are-we-ready-to-govern-it.html</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>S13</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Cedar Report / Newswire / Fintech.ca / RBCCM</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Canadian banks agentic AI (RBC, TD, Scotia, BMO, CIBC)</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>https://www.cedarreport.com/guides/how-canadian-banks-are-using-ai-in-2026-rbc-td-bmo-and-more</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>S14</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>The Financial Brand / Capital One / TechCrunch / NVIDIA On-Demand</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Capital One Chat Concierge + agentic AI</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>https://thefinancialbrand.com/news/banking-products/capital-ones-chat-concierge-puts-agentic-ai-on-car-dealers-websites-187128</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>S15</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Truist IR / PNC / American Banker / FinancialContent</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Truist receivables, PNC working capital, US Bank developer assistant</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>https://ir.truist.com/2026-02-03-Truist-launches-AI-enabled-receivables-platform-to-accelerate-cash-application-and-minimize-exceptions</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>S16</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>TheLetterTwo / Digital Commerce 360 / American Banker / ClearingPost / adwaitx</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Visa Intelligent Commerce Connect, Mastercard Agent Suite/Pay</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>https://thelettertwo.com/2026/04/08/visa-wants-to-be-the-payment-rail-for-the-agentic-economy</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>S17</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Digital Commerce 360 / Fortune</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>American Express ACE developer kit + Agent Purchase Protection</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>https://www.digitalcommerce360.com/2026/04/14/american-express-agentic-commerce-developer-kit-purchase-protection/</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>S18</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>PayPal Newsroom / PayPal Tech Blog / PayPal.ai</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>PayPal Agent Ready, Store Sync, MCP servers</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>https://newsroom.paypal-corp.com/2025-10-28-PayPal-Launches-Agentic-Commerce-Services-to-Power-AI-Driven-Shopping</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>S19</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Stripe blog / Stripe docs / agenticcommerce.expert / GitHub</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Stripe Agentic Commerce Suite + ACP</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>http://www.stripe.com/blog/agentic-commerce-suite</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>S20</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Anthropic / Economic Times / ETCFO / ClaudeReadiness</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Claude for Financial Services + Goldman Sachs deployment</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>https://www.anthropic.com/solutions/financial-services</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>S21</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Adyen / Major Matters</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Adyen agentic-commerce strategy + Universal Token Vault</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adyen.com/knowledge-hub/adyen-joins-agentic-ai-foundation</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>S22</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>FIS press / Temenos</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>FIS agentic commerce platform + Temenos FCM AI Agent</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>https://www.fisglobal.com/about-us/media-room/press-release/2026/fis-launches-industry-first-ai-transaction-platform-to-help-banks-lead</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>S23</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Synchrony Newsroom</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Synchrony agentic-commerce strategy</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>https://www.synchrony.com/contenthub/insights/blog-post-by-mike-storiale.html</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>S24</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Markets Insider (Bernstein note)</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Bernstein bullish on Fiserv, Block, Adyen for agentic commerce</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>https://markets.businessinsider.com/news/stocks/fiserv-block-and-adyen-here-s-why-bernstein-is-bullish-on-these-3-fintech-stocks-1035185068</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>S25</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>OpenAI / ad-hoc-news / myaskai / Klarna</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Klarna AI assistant plus 2026 reversal coverage</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>https://www.ad-hoc-news.de/boerse/news/ueberblick/klarna-s-ai-pivot-reversing-course-after-customer-service-setbacks/69026000</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>S26</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>FStech / FinTech Weekly / Marcel van Oost / Fintyle</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Nubank, Revolut AIR, Starling Assistant, Monzo coverage</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>https://www.fintechweekly.com/news/revolut-air-ai-assistant-uk-customers-launch-2026</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>S27</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Brex.ai / Ramp blog / Stack-ai</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Brex Agents + Ramp agentic AP and expense</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>https://www.brex.ai/</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>S28</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>SiliconANGLE / aihaberleri / theoutpost / stacks.ai / uktech.news</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>2026 agentic-AI fintech funding rounds (Slash, Dyna.Ai, Stacks, EnFi, Ralio)</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>https://siliconangle.com/2026/04/16/slash-raises-100m-1-4b-valuation-expand-ai-powered-banking-platform-online-businesses/</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>S29</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Hebbia / V7Labs / CB Insights</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Hebbia, Glean, Harvey product + funding profiles</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>https://www.hebbia.com/blog/whats-new-april-disclosure-2026</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>S30</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Fenergo / Bretton / Stack-ai / dev.to</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>Compliance / financial-crime agentic vendors</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>https://fenergo.com/agentic-ai-agents</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>S31</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>KX / NVIDIA On-Demand / NVIDIA blog</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>KX agentic AI blueprints + Capital One GTC 2026 talk + NVIDIA FS survey</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>https://kx.com/news-room/kx-launches-agentic-ai-blueprints-powered-by-nvidia-at-gtc-2026-featuring-a-capital-markets-research-assistant-and-trading-signal-agent/</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>S32</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>Coinbase / Linux Foundation / Crossmint / aiagentstore</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>x402 protocol launch + Skyfire / Crossmint comparison</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>https://blog.crossmint.com/what-is-x402/</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>S33</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Microsoft Learn / Microsoft Industry Blog / myabt / Microsoft Adoption</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Microsoft Finance Agents + Agent 365 + Copilot for FS</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>https://www.microsoft.com/en-us/industry/blog/financial-services/banking/2026/02/26/the-agentic-moment-in-banking-a-blueprint-for-better-customer-experiences/</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>S34</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>Google Cloud / Promevo / ScaleByTech</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>Gemini Enterprise (Agentspace) for banking</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>https://cloud.google.com/products/agentspace</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>S35</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>Google / Adyen / Crossmint</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>Universal Commerce Protocol (UCP) + Agent Payments Protocol (AP2)</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>https://www.crossmint.com/learn/agentic-payments-protocols-compared</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>S36</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>OpenAI / OpenAI Developers / Ekamoira</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>ChatGPT Instant Checkout + Agentic Commerce Protocol</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>https://openai.com/index/buy-it-in-chatgpt/</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>S37</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>Salesforce / Vantage Point</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>Agentforce for Financial Services</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>https://www.salesforce.com/financial-services/artificial-intelligence/</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
+          <t>S1–S37</t>
         </is>
       </c>
     </row>

</xml_diff>